<commit_message>
Agregar FUENTE.md, paper de CONDA y modelado lineal (filtro, logistica y SVM)
- FUENTE.md con URL, institucion y huellas SHA-256 de CONDA y Jigsaw
- Paper de CONDA (Weld et al. 2021) en Fuentes y en la matriz (fila 51)
- Proyecto/Modelado: filtro de palabras, regresion logistica y SVM lineal por
  fuente, con split por partida en CONDA, tabla con las dos tasas y RESULTADOS.md
</commit_message>
<xml_diff>
--- a/Articulos/Revision/Matriz_de_Revision.xlsx
+++ b/Articulos/Revision/Matriz_de_Revision.xlsx
@@ -2774,18 +2774,50 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="30" customHeight="1">
+    <row r="52" ht="96" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="n"/>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Weld, Huang, Lee, Zhang, Wang, Guo, Long, Poon &amp; Han, 2021</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>CONDA: a CONtextual Dual-Annotated dataset for in-game toxicity understanding and detection</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Findings of ACL-IJCNLP 2021</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2106.06213</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Los datasets de toxicidad analizan cada mensaje aislado, sin el contexto de la conversacion ni las pistas de las palabras del juego; faltaba un conjunto de chat de videojuego que permita detectar toxicidad explicita e implicita</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Dataset de 44,869 mensajes de 12,152 conversaciones en 1,921 partidas de Dota 2, con anotacion dual: intencion del mensaje (E explicita, I implicita, A accion, O otro) etiquetada a mano por jugadores, y etiqueta por palabra generada con lexicones. Se evaluan cinco modelos (RNN-NLU, Slot-gated, Inter-BiLSTM, Capsule NN, Joint BERT) con split 0.6/0.2/0.2</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Joint BERT fue el mejor: exactitud por mensaje de 0.921 y F1 por clase de E 0.872, I 0.768, A 0.800 y O 0.954; la clase implicita es la mas dificil. La clase O es 73.9% de los mensajes y las toxicas (E+I) 19.7%. Acuerdo entre anotadores jugadores: kappa de Fleiss 0.785. Entrenado en CONDA y probado en otros datasets, la exactitud va de 0.669 (FoxNews) a 0.875 (StormfrontWS)</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>POR COMPLETAR (quien lo lea)</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="2" t="n">

</xml_diff>

<commit_message>
Matriz de revision con los 4 articulos nuevos (33, 41, 47, 50) y BiGRU por fuente
- Matriz_de_Revision.xlsx: filas 33, 41, 47 y 50 reemplazadas (los PDFs anteriores ya no estaban disponibles).
- 02_bigru.py: BiGRU con embeddings desde cero, 3 semillas, mismos splits y metricas que los lineales.
- Resultados/resultados_bigru.csv y .md.
</commit_message>
<xml_diff>
--- a/Articulos/Revision/Matriz_de_Revision.xlsx
+++ b/Articulos/Revision/Matriz_de_Revision.xlsx
@@ -1970,37 +1970,37 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Taulé, Nofre, Bargiela &amp; Bonet, 2024</t>
+          <t>Davidson, Warmsley, Macy &amp; Weber, 2017</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>NewsCom-TOX: a corpus of comments on news articles annotated for toxicity in Spanish</t>
+          <t>Automated Hate Speech Detection and the Problem of Offensive Language</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Language Resources and Evaluation 58(4)</t>
+          <t>ICWSM 2017 (AAAI)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s10579-023-09711-x</t>
+          <t>https://doi.org/10.1609/icwsm.v11i1.14955</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Faltan recursos anotados para detectar toxicidad en espanol, sobre todo comentarios con contenido racista y xenofobo en noticias</t>
+          <t>Los metodos basados en diccionarios de palabras marcan como odio cualquier mensaje con una palabra ofensiva, sin distinguir entre discurso de odio y lenguaje simplemente vulgar</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Corpus anotado manualmente en varios niveles con categorias binarias (postura, objetivo, estereotipo, sarcasmo, burla, insulto, lenguaje inapropiado, agresividad e intolerancia), considerando el hilo completo y la noticia con sus imagenes</t>
+          <t>Lexico de odio de Hatebase para recolectar tweets, etiquetado por crowdsourcing en 3 clases (odio, ofensivo, ninguno) y clasificador multiclase de regresion logistica con regularizacion L2</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Corpus de 4,359 comentarios en espanol publicados en respuesta a 21 noticias sobre inmigracion, anotados con 9 categorias linguisticas que permiten asignar un nivel de toxicidad a cada comentario; sirvio como dataset oficial de la tarea DETOXIS de IberLEF 2021</t>
+          <t>Sobre 24,802 tweets etiquetados (solo 5% marcados como odio por mayoria), el modelo obtuvo precision global de 0.91, recall de 0.90 y F1 de 0.90; en la clase de odio la precision cayo a 0.44 y el recall a 0.61</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2324,43 +2324,43 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="96" customHeight="1">
+    <row r="42" ht="110" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Salminen, Hopf, Chowdhury, Jung, Almerekhi &amp; Jansen, 2020</t>
+          <t>Pavlopoulos, Sorensen, Dixon, Thain &amp; Androutsopoulos, 2020</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Developing an online hate classifier for multiple social media platforms</t>
+          <t>Toxicity Detection: Does Context Really Matter?</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Human-centric Computing and Information Sciences 10(1)</t>
+          <t>ACL 2020</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1186/s13673-019-0205-6</t>
+          <t>https://doi.org/10.18653/v1/2020.acl-main.396</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Los clasificadores de odio se entrenan con datos de una sola plataforma y no se sabe si generalizan a otras</t>
+          <t>Casi todos los datasets de toxicidad etiquetan comentarios de forma aislada, asumiendo que el hilo de conversacion no cambia el juicio</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Recoleccion multiplataforma de comentarios etiquetados y comparacion de Regresion Logistica, Naive Bayes, SVM, XGBoost y redes neuronales con representaciones Bag-of-Words, TF-IDF, Word2Vec, BERT y sus combinaciones</t>
+          <t>Re-anotacion de comentarios de paginas de discusion de Wikipedia en dos condiciones (con y sin contexto: titulo del hilo y comentario previo), sobre subconjuntos de 250 y 10,000 comentarios, mas clasificadores sensibles al contexto</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Sobre 197,566 comentarios de YouTube, Reddit, Wikipedia y Twitter (20% etiquetados como odio), XGBoost con todos los rasgos obtuvo el mejor resultado con F1 de 0.92; los rasgos derivados de BERT fueron los mas influyentes en la prediccion</t>
+          <t>El 5% de los comentarios cambio de etiqueta al mostrar el contexto (diferencia estadisticamente significativa, P &lt; .01), pero ningun clasificador sensible al contexto mejoro el desempeno frente a los que ignoran el contexto</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2594,43 +2594,43 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="96" customHeight="1">
+    <row r="48" ht="123" customHeight="1">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Almerekhi, Kwak, Salminen &amp; Jansen, 2022</t>
+          <t>Fortuna, Soler &amp; Wanner, 2020</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Investigating toxicity changes of cross-community redditors from 2 billion posts and comments</t>
+          <t>Toxic, Hateful, Offensive or Abusive? What Are We Really Classifying? An Empirical Analysis of Hate Speech Datasets</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>PeerJ Computer Science</t>
+          <t>LREC 2020 (ELRA)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.7717/peerj-cs.1059</t>
+          <t>https://aclanthology.org/2020.lrec-1.838</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>No se sabia si la toxicidad es un rasgo estable de la persona o si el mismo usuario ajusta su conducta segun las normas de cada comunidad</t>
+          <t>Los datasets de discurso de odio usan categorias y definiciones distintas para conceptos equivalentes, lo que dificulta compararlos y combinarlos</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Dataset etiquetado por crowdsourcing usado para afinar un modelo BERT, aplicado despues a todo el historial de Reddit de 2005 a 2020 para medir cambios de toxicidad por usuario, por comunidad y en el tiempo</t>
+          <t>Analisis empirico de 6 datasets publicos en 2 experimentos: (1) representar las clases como vectores FastText para medir su similitud dentro y entre datasets; (2) evaluar los datasets con el clasificador de toxicidad de la Perspective API</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Con 10,083 comentarios etiquetados, BERT alcanzo 91.27% de exactitud y AUC de 0.963; al aplicarlo a 87,376,912 publicaciones y 2,205,581,786 comentarios se encontro que 16.11% de los usuarios publican posts toxicos y que 30.68% (posts) y 81.67% (comentarios) cambian su nivel de toxicidad entre comunidades</t>
+          <t>Se analizaron 6 datasets publicos en 2 experimentos; el desempeno de la Perspective API vario segun la categoria y el dataset, y se concluye que se usan muchas definiciones distintas para conceptos equivalentes, por lo que la mayoria de los datasets publicos son incompatibles. POR COMPLETAR: cifras de desempeno por dataset (leer el articulo completo)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2729,43 +2729,43 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="96" customHeight="1">
+    <row r="51" ht="136" customHeight="1">
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Soral, Bilewicz &amp; Winiewski, 2018</t>
+          <t>Schöpke-Gonzalez, Wu, Kumar, Resnick &amp; Hemphill, 2023</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Exposure to hate speech increases prejudice through desensitization</t>
+          <t>How We Define Harm Impacts Data Annotations: Explaining How Annotators Distinguish Hateful, Offensive, and Toxic Comments</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Aggressive Behavior 44(2)</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/ab.21737</t>
+          <t>https://doi.org/10.48550/arXiv.2309.15827</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Se desconocia el mecanismo por el cual la exposicion frecuente a discurso de odio en linea termina aumentando el prejuicio hacia los grupos atacados</t>
+          <t>Los datasets de dano en linea suelen tratar "odioso", "ofensivo" y "toxico" como sinonimos, sin saber si los anotadores los distinguen ni por que</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Tres estudios enmarcados en el Modelo General de Agresion: dos encuestas representativas a nivel nacional y un experimento con entrenamiento de desensibilizacion frente a un grupo de control</t>
+          <t>Analisis de contenido y regresion sobre 3,481 comentarios de Reddit, Twitter y YouTube anotados por 5 trabajadores de MTurk cada uno como odiosos, ofensivos o toxicos; codebook propio aplicado a 909 comentarios, diagramas de Venn y razon de informacion mutua (MIR)</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Con muestras de N = 1,007 y N = 682 en las encuestas y N = 76 en el experimento, la menor sensibilidad al discurso de odio actuo como mediador entre la exposicion frecuente y el prejuicio; los participantes desensibilizados evaluaron peor a las victimas que el grupo de control (paginas 136-146)</t>
+          <t>De 823 comentarios dirigidos, 17.98% fueron odiosos, 34.14% ofensivos y 35.00% toxicos; "odioso" es el concepto mas distinto (MIR de 0.292 a 0.422 en los pares que lo incluyen) y ofensivo/toxico se parecen mas (MIR de ofensivo a toxico: 0.741); el efecto del anotador fue el predictor mas fuerte (razon de momios 5.75 en odioso, 4.69 en ofensivo y 7.30 en toxico)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Matriz de revision de 60 articulos sin repetidos y fuentes ordenadas
- Matriz_de_Revision.xlsx: 60 filas. Se completaron las filas 52 a 60 con articulos leidos (con cifras) y se reemplazaron las filas 33 y 41, que repetian a las 21 y 26 (Davidson 2017 y Pavlopoulos 2020, misma DOI), por Xenos et al. 2021 y Stoop et al. 2019. Se corrigio el No.50 (porcentajes de ofensivo y toxico) y el No.47 (sin cifras por dataset: el articulo las muestra solo en una figura).

- Fuentes/: los 60 PDFs en una sola carpeta, numerados como la matriz (01_ a 60_), cada uno verificado contra el titulo de su fila. Se agrego INDICE.md. Se quitaron 2 duplicados y un archivo vacio.

- FUENTE.md: quien y cuando descargo CONDA y Jigsaw.
</commit_message>
<xml_diff>
--- a/Articulos/Revision/Matriz_de_Revision.xlsx
+++ b/Articulos/Revision/Matriz_de_Revision.xlsx
@@ -1970,42 +1970,42 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Davidson, Warmsley, Macy &amp; Weber, 2017</t>
+          <t>Xenos, Pavlopoulos, Androutsopoulos, Dixon, Sorensen &amp; Laugier, 2021</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Automated Hate Speech Detection and the Problem of Offensive Language</t>
+          <t>Toxicity Detection can be Sensitive to the Conversational Context</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>ICWSM 2017 (AAAI)</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1609/icwsm.v11i1.14955</t>
+          <t>https://doi.org/10.48550/arXiv.2111.10223</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Los metodos basados en diccionarios de palabras marcan como odio cualquier mensaje con una palabra ofensiva, sin distinguir entre discurso de odio y lenguaje simplemente vulgar</t>
+          <t>Los datasets de toxicidad casi no tienen comentarios cuya toxicidad dependa del mensaje anterior, asi que los detectores entrenados con ellos ignoran el contexto y fallan cuando si importa</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Lexico de odio de Hatebase para recolectar tweets, etiquetado por crowdsourcing en 3 clases (odio, ofensivo, ninguno) y clasificador multiclase de regresion logistica con regularizacion L2</t>
+          <t>Dataset propio de 10,000 comentarios de Civil Comments con dos etiquetas: de anotadores que vieron el mensaje anterior como contexto y de anotadores que no lo vieron. Nueva tarea de estimacion de la sensibilidad al contexto, evaluada con regresion lineal, SVR, bosque aleatorio y un BERT de regresion (BERTr), con aumento de datos por destilacion de conocimiento; ademas se prueba Perspective API sin ajuste</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Sobre 24,802 tweets etiquetados (solo 5% marcados como odio por mayoria), el modelo obtuvo precision global de 0.91, recall de 0.90 y F1 de 0.90; en la clase de odio la precision cayo a 0.44 y el recall a 0.61</t>
+          <t>En 66.1% de los comentarios la toxicidad no cambio al mostrar el contexto; en el resto subio en 9.6% (960 comentarios) y bajo en 24.3% (2,408), y al binarizar las etiquetas 94.7% no cambia. El mejor estimador de sensibilidad al contexto fue BERTr, con AUPR de 42.01 y AUC de 80.46, contra 30.11 y 71.67 de la regresion lineal y 12.69 y 50.00 de la linea base del promedio (promedio de 3 particiones). El error de Perspective API crece con la sensibilidad al contexto del comentario</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Maurizio López</t>
+          <t>Carlos Saavedra</t>
         </is>
       </c>
     </row>
@@ -2330,42 +2330,42 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Pavlopoulos, Sorensen, Dixon, Thain &amp; Androutsopoulos, 2020</t>
+          <t>Stoop, Kunneman, van den Bosch &amp; Miller, 2019</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Toxicity Detection: Does Context Really Matter?</t>
+          <t>Detecting harassment in real-time as conversations develop</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ACL 2020</t>
+          <t>Third Workshop on Abusive Language Online (ACL 2019)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://doi.org/10.18653/v1/2020.acl-main.396</t>
+          <t>https://doi.org/10.18653/v1/W19-3503</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Casi todos los datasets de toxicidad etiquetan comentarios de forma aislada, asumiendo que el hilo de conversacion no cambia el juicio</t>
+          <t>Casi todos los detectores de acoso evaluan conversaciones ya terminadas, pero para intervenir durante una partida (advertir, silenciar o expulsar) hay que detectar al jugador tomando en cuenta solo lo dicho hasta ese momento</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Re-anotacion de comentarios de paginas de discusion de Wikipedia en dos condiciones (con y sin contexto: titulo del hilo y comentario previo), sobre subconjuntos de 250 y 10,000 comentarios, mas clasificadores sensibles al contexto</t>
+          <t>Marco HaRe: red recurrente con embeddings de 300 dimensiones, dos GRU bidireccionales de 16 unidades y dos capas densas de 256, entrenada con 4,000 conversaciones de League of Legends y evaluada con 1,000 (5,000 conversaciones de 48,512 jugadores, con 186.77 mensajes por conversacion en promedio; 10.3% de los jugadores fueron marcados como toxicos por el Tribunal de Riot Games). Se mide precision, recall y F1 por jugador a lo largo de la conversacion con distintos umbrales de confianza</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>El 5% de los comentarios cambio de etiqueta al mostrar el contexto (diferencia estadisticamente significativa, P &lt; .01), pero ningun clasificador sensible al contexto mejoro el desempeno frente a los que ignoran el contexto</t>
+          <t>El recall sube y la precision baja conforme avanza la conversacion; el umbral de confianza con mejor F1 debe empezar bajo y subir durante la conversacion, y sube mas despacio cuanto mayor es el conjunto de entrenamiento. El articulo muestra estos resultados en graficas (figuras 3 a 6) y no da cifras de precision ni de recall en el texto</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Victor Salazar</t>
+          <t>Carlos Saavedra</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Se analizaron 6 datasets publicos en 2 experimentos; el desempeno de la Perspective API vario segun la categoria y el dataset, y se concluye que se usan muchas definiciones distintas para conceptos equivalentes, por lo que la mayoria de los datasets publicos son incompatibles. POR COMPLETAR: cifras de desempeno por dataset (leer el articulo completo)</t>
+          <t>Se analizaron 6 datasets publicos (Waseem, Davidson, Amievalita, Hateval, TRAC y Toxkaggle). Con la Perspective API (en Toxkaggle se uso una muestra de 20%, 31,914 mensajes) el F1 vario mucho por categoria: mejor en toxicidad y ofensivo, despues obsceno, insulto, misoginia-sexismo y discurso de odio; peor en agresion, racismo, toxico severo y amenaza. Para una misma categoria tambien varia entre datasets (discurso de odio: mayor F1 en Davidson que en Hateval; toxicidad y agresion: mayor en Davidson que en Toxkaggle). Las 2 primeras componentes principales de los centroides de clase explican 92% de la varianza (77.5% + 14.5%). Se concluye que se usan muchas definiciones distintas para conceptos equivalentes, por lo que la mayoria de los datasets publicos son incompatibles. Nota: el articulo muestra los F1 solo en la Figura 3, sin valores numericos</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>De 823 comentarios dirigidos, 17.98% fueron odiosos, 34.14% ofensivos y 35.00% toxicos; "odioso" es el concepto mas distinto (MIR de 0.292 a 0.422 en los pares que lo incluyen) y ofensivo/toxico se parecen mas (MIR de ofensivo a toxico: 0.741); el efecto del anotador fue el predictor mas fuerte (razon de momios 5.75 en odioso, 4.69 en ofensivo y 7.30 en toxico)</t>
+          <t>De 823 comentarios dirigidos, 17.98% fueron odiosos, 34.99% ofensivos y 34.14% toxicos; "odioso" es el concepto mas distinto (MIR de 0.292 a 0.422 en los pares que lo incluyen) y ofensivo/toxico se parecen mas (MIR de ofensivo a toxico: 0.741); el efecto del anotador fue el predictor mas fuerte (razon de momios 5.75 en odioso, 4.69 en ofensivo y 7.30 en toxico)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>POR COMPLETAR (quien lo lea)</t>
+          <t>Carlos Saavedra</t>
         </is>
       </c>
     </row>
@@ -2823,118 +2823,406 @@
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Andariefli, Leonard, Dewanto &amp; Novika, 2025</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Comparative analysis of two-class and multi-class toxicity detection using multi-source gaming chat data</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Procedia Computer Science 269</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.procs.2025.09.025</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>El chat toxico en juegos competitivos como Dota 2 degrada la experiencia de los jugadores, y no se sabia que arquitectura de aprendizaje profundo funciona mejor con mensajes cortos y muy desbalanceados</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Corpus de 5,469 mensajes de chat de Dota 2 que combina 2 datasets publicos (Kaggle y Hugging Face) en 3 clases (no toxico 2,987; toxico 926; muy toxico 1,556), embeddings GloVe de 100 dimensiones con relleno a 150 tokens, y comparacion de una LSTM contra una CNN 1D (kernel 5, max pooling global), ambas con Adam</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>La LSTM solo predijo la clase mayoritaria: exactitud de 53.4%, F1 de 0.70 en no toxico y 0.00 en las otras dos clases. La CNN logro exactitud de 79.9% y F1 de 0.91 (no toxico), 0.64 (toxico) y 0.66 (muy toxico). Los autores advierten que la exactitud global engana por el desbalance</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Beddiar, Jahan &amp; Oussalah, 2021</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Data expansion using back translation and paraphrasing for hate speech detection</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Online Social Networks and Media 24</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.osnem.2021.100153</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Entrenar modelos profundos para detectar discurso de odio y ciberacoso requiere muchos datos etiquetados de calidad, que casi siempre faltan</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Aumento de datos con retrotraduccion (codificador-decodificador) y parafraseo (transformer con mezcla de expertos), que duplican y casi decuplican el dataset (20 veces al combinarlos); embeddings FastText y clasificacion con CNN y LSTM (la CNN tambien se compara con regresion logistica y Naive Bayes sobre n-gramas de caracteres); evaluado en 5 datasets publicos: AskFm, Formspring, Warner y Waseem, OLID y comentarios toxicos de Wikipedia</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Con CNN y retrotraduccion + parafraseo, el F1 pasa de 95.3% a 99.4% en Wikipedia, de 89.0% a 99.3% en Warner y Waseem y de 71.0% a 94.5% en OLID. El mejor recall (99.7%) y precision (99.6%) se dieron en Warner y Waseem expandido</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Sengun, Santos, Salminen, Jung &amp; Jansen, 2022</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Do players communicate differently depending on the champion played? Exploring the Proteus effect in League of Legends</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Technological Forecasting &amp; Social Change 177</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.techfore.2022.121556</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>No se sabia si el personaje que usa un jugador (efecto Proteo) cambia su forma de comunicarse en el chat: cuanto escribe (vocalidad), que tan negativo es (valencia) y que tan toxico es</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>13.6 millones de mensajes de chat de League of Legends y 136 campeones descritos con variables objetivas (datos del desarrollador y codificacion semiotica) y subjetivas (calificaciones de 15 trabajadores de crowdsourcing por campeon); regresiones jerarquicas para vocalidad, valencia y toxicidad (frecuencia de palabras toxicas), y comparacion dentro y entre campeones con 1,000 a 5,000 jugadores que usaron mas de un campeon</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Con solo variables objetivas el modelo explica 29.7% de la varianza de la vocalidad, 54.3% de la valencia y 60% de la toxicidad; las subjetivas solo mejoran significativamente la valencia (+9.9 puntos, p &lt; .05). Los Fighters son mas toxicos que los Tanks (b = 0.231, p &lt; .001) y los Support menos (b = -0.341, p &lt; .001). En 1,000 jugadores que usaron varios campeones, la toxicidad cambia mas entre campeones que entre partidas (t(999) = 4.439, p &lt; .001)</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Zsila, Orosz &amp; Demetrovics, 2025</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Reducing toxic behaviors in the gaming community: A social-psychological intervention with lasting effects</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Computers in Human Behavior 176</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.chb.2025.108827</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>La toxicidad entre jugadores reduce el disfrute y el bienestar, y faltaba evidencia experimental de que una intervencion breve disminuya las reacciones desadaptativas ante ella</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Ensayo controlado aleatorizado preregistrado con 722 jugadores (372 en tratamiento y 350 en control): el tratamiento leia testimonios de pares sobre estrategias adaptativas contra la toxicidad y el control, sobre circunstancias externas disruptivas; mediciones antes, justo despues y un mes despues; pruebas t de Welch con g de Hedges</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Justo despues, el grupo de tratamiento mostro menos rumiacion (p = .046, g = 0.17), menos reacciones desadaptativas (p = .006, g = 0.24) y mas reacciones adaptativas (p = .003, g = 0.26). Un mes despues solo se mantuvo la reduccion de reacciones desadaptativas (p = .030, g = 0.30); no hubo diferencias en disfrute, involucramiento en conductas toxicas ni desinhibicion toxica (p = .731, .240 y .690)</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
-      <c r="I57" s="2" t="n"/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Thompson, Leung, Blair &amp; Taboada, 2017</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Sentiment analysis of player chat messaging in the video game StarCraft 2: Extending a lexicon-based model</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Knowledge-Based Systems 137</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.knosys.2017.09.022</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Hacen falta herramientas portables que estimen el sentimiento y detecten toxicidad en el chat de videojuegos sin entrenar un modelo nuevo para cada dominio</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Extension del extractor de sentimiento basado en lexicon SO-CAL con entradas de diccionario propias del juego, bloqueo de emoticonos y un parametro de repeticion, aplicado a los mensajes de 1,000 partidas de StarCraft 2 evaluadas por jueces humanos y verificado con 2,025 partidas adicionales</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>El mejor modelo (NoRepBlock) tuvo 70% de exactitud (desv. 4%) en 3 clases de sentimiento con muestras balanceadas: 85% en partidas con 4 mensajes o menos y 71% en las de 5 o mas. Los modelos con otros diccionarios no pasaron de 50.7%, casi igual que predecir siempre positivo (50.4%). Como detector de toxicidad tuvo 33% de aciertos y 0.7% de falsas alarmas; en las 2,025 partidas nuevas marco 21 como toxicas y 10 lo eran (precision de 47.6%, contra 56.2% esperada)</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Yang, Grenon-Godbout &amp; Rabbany, 2023</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Towards Detecting Contextual Real-Time Toxicity for In-Game Chat</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Findings of EMNLP 2023</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.18653/v1/2023.findings-emnlp.663</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Los modelos de toxicidad revisan cada linea de chat aislada, sin el historial de la partida ni datos del jugador, y no funcionan bien en tiempo real en chats de videojuegos</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>ToxBuster: BERT afinado que clasifica cada linea de chat por clase de toxicidad usando el historial de chat (alcance personal, de equipo, global o de moderador) y metadatos (equipo, tipo de chat, jugador); evaluado en chats de Rainbow Six Siege (95,612 lineas), For Honor (99,371) y DOTA 2 (62,483), y en Civil Comments de Jigsaw (131,319), contra Cleanspeak, Perspective API y Detoxify. Version ampliada del trabajo de la fila 2 (otros autores y datos nuevos)</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>F1 ponderado de ToxBuster de 83.25 en Rainbow Six Siege, 85.09 en For Honor, 84.53 en DOTA 2 y 95.47 en Civil Comments; los baselines (que solo clasifican toxico/no toxico) obtuvieron 36.81-40.48 en Rainbow Six Siege y 1.95-5.75 en DOTA 2. En Rainbow Six Siege el F1 sube de 77.36 sin historial a 78.89 con el historial del propio jugador, 81.30 con el del equipo y 81.70 con el global. Marca 82.1% de los jugadores reportados por chat con 90.0% de precision</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
-      <c r="I59" s="2" t="n"/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Nejadgholi &amp; Kiritchenko, 2020</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>On Cross-Dataset Generalization in Automatic Detection of Online Abuse</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>WOAH 2020 (4th Workshop on Online Abuse and Harms)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2010.07414</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Los detectores de abuso se evaluan con datos parecidos a los de entrenamiento, pero en la practica se aplican a datos con otros temas y otra distribucion de clases, y no se sabia cuanto de la caida al cambiar de dataset se debe al sesgo de tema</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>BERT con capa lineal (lote de 16, tasa de aprendizaje 2e-5, 2 epocas) entrenado con los comentarios de Wikipedia (Wiki Detox) y evaluado fuera de dominio con un conjunto que combina los datasets de Twitter de Waseem y de Founta; modelado de temas no supervisado (20 temas) para separar los comentarios en 3 categorias y probar quitando los de temas propios de Wikipedia</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Fuera de dominio el F1 macro es alto (0.89), pero la exactitud por clase varia mucho: 0.94 en Founta-Abusive, 0.62 en Founta-Hateful, 0.26 en Waseem-Sexist y 0.35 en Waseem-Racist. Los temas propios de Wikipedia son 54% de los comentarios; quitar los ejemplos normales de esos temas sube la exactitud en todas las clases (por ejemplo Founta-Hateful de 0.62 a 0.67 y Waseem-Sexist de 0.26 a 0.30) y el F1 macro fuera de dominio de 0.89 a 0.91, sin bajar el de dominio (0.89)</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="n"/>
-      <c r="I60" s="2" t="n"/>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Piedras, Rosenblatt &amp; Wilkins, 2022</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Critical Perspectives: A Benchmark Revealing Pitfalls in PerspectiveAPI</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>NLP for Positive Impact (EMNLP 2022 workshop)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arXiv.2301.01874</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>PerspectiveAPI se usa para medir toxicidad y declara resultados muy buenos, pero no se habia probado con toxicidad sutil ni con groserias usadas sin mala intencion</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark SASS con 250 ejemplos creados a mano en 10 categorias de toxicidad (8 de falsos negativos, 1 de falsos positivos y 1 neutral), cada uno con una calificacion humana de toxicidad; clasificacion binaria con PerspectiveAPI y con GPT-3 en prompts zero-shot, one-shot y few-shot. Los ejemplos filtrados se crearon para obtener puntajes bajos en PerspectiveAPI</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>PerspectiveAPI: precision 0.26, recall 0.05 y F1 0.08; GPT-3 zero-shot F1 0.31, one-shot 0.19 y few-shot 0.61 (precision 0.73, recall 0.52). En los 18 ejemplos no toxicos que contienen groserias, PerspectiveAPI los califico todos como toxicos y GPT-3 few-shot el 83%, lo que sugiere que los modelos memorizan las groserias en lugar de entender la intencion</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
-      <c r="I61" s="2" t="n"/>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Tereshchenko &amp; Hamalainen, 2025</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Efficient Toxicity Detection in Gaming Chats: A Comparative Study of Embeddings, Fine-Tuned Transformers and LLMs</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Journal of Data Mining and Digital Humanities (NLP4DH)</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.46298/jdmdh.16280</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>La moderacion manual de chats de videojuegos no escala y no se sabia que enfoque (clasificadores con embeddings, LLMs con prompts, modelos afinados o RAG) da el mejor balance entre exactitud, velocidad y costo</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Entrenamiento con Jigsaw (159,571 comentarios) y prueba en GOSU.ai, chat de Dota 2 (147,842 mensajes: 68.2% limpios, 19.7% toxicidad leve y 12.1% fuerte); compara SVM y regresion logistica con SGD sobre embeddings, GPT-3.5 y GPT-4 zero-shot y few-shot (100 mensajes), RAG, y modelos afinados (DialoGPT y DistilBERT con 2,613 mensajes de GOSU.ai); mide exactitud, latencia y costo, y propone un sistema hibrido de moderacion</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Entrenados en Jigsaw y probados en GOSU.ai: SVM con exactitud 0.808, recall 0.612, F1 0.741 y ROC-AUC 0.900, y regresion logistica con F1 0.711. GPT-4 zero-shot, el mejor LLM, con exactitud 0.910 y F1 0.866 (unos 1.1 s por mensaje); GPT-3.5 zero-shot con F1 0.720 (unos 700 ms). DialoGPT afinado con exactitud 0.674 y F1 0.586; DistilBERT afinado con GOSU.ai con exactitud 0.943 y F1 0.936 en su subconjunto de prueba, que los autores consideran el mejor balance exactitud-costo</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Saavedra</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1"/>
   </sheetData>

</xml_diff>